<commit_message>
Add Tercier research, models, and supporting materials
</commit_message>
<xml_diff>
--- a/tercier-financial-model.xlsx
+++ b/tercier-financial-model.xlsx
@@ -21,7 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity Analysis" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001" forceFullCalc="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
 </file>
 
@@ -2958,8 +2958,9 @@
           <t>Founder salary (EUR/month)</t>
         </is>
       </c>
-      <c r="B75" s="144" t="n">
-        <v>4395.604395604396</v>
+      <c r="B75" s="144">
+        <f>B74/(12*$B$6)</f>
+        <v/>
       </c>
       <c r="C75" s="127" t="n"/>
       <c r="D75" s="136" t="inlineStr">
@@ -8391,8 +8392,9 @@
       <c r="D5" s="236" t="n">
         <v>4138544</v>
       </c>
-      <c r="E5" s="237" t="n">
-        <v>-0.194</v>
+      <c r="E5" s="237">
+        <f>D5/31537836</f>
+        <v/>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="125">
@@ -8412,8 +8414,9 @@
       <c r="D6" s="239" t="n">
         <v>-6124507</v>
       </c>
-      <c r="E6" s="240" t="n">
-        <v>0.131</v>
+      <c r="E6" s="240">
+        <f>D6/31537836</f>
+        <v/>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="125">
@@ -8433,8 +8436,9 @@
       <c r="D7" s="241" t="n">
         <v>4578819</v>
       </c>
-      <c r="E7" s="242" t="n">
-        <v>0.145</v>
+      <c r="E7" s="242">
+        <f>D7/31537836</f>
+        <v/>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="125">
@@ -8454,8 +8458,9 @@
       <c r="D8" s="243" t="n">
         <v>-5337817</v>
       </c>
-      <c r="E8" s="244" t="n">
-        <v>-0.169</v>
+      <c r="E8" s="244">
+        <f>D8/31537836</f>
+        <v/>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="125">
@@ -8475,8 +8480,9 @@
       <c r="D9" s="241" t="n">
         <v>4234861</v>
       </c>
-      <c r="E9" s="242" t="n">
-        <v>0.134</v>
+      <c r="E9" s="242">
+        <f>D9/31537836</f>
+        <v/>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="125">
@@ -8496,8 +8502,9 @@
       <c r="D10" s="243" t="n">
         <v>-4503740</v>
       </c>
-      <c r="E10" s="244" t="n">
-        <v>-0.143</v>
+      <c r="E10" s="244">
+        <f>D10/31537836</f>
+        <v/>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="125">
@@ -8517,8 +8524,9 @@
       <c r="D11" s="241" t="n">
         <v>506082</v>
       </c>
-      <c r="E11" s="242" t="n">
-        <v>0.016</v>
+      <c r="E11" s="242">
+        <f>D11/31537836</f>
+        <v/>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="125">
@@ -8538,8 +8546,9 @@
       <c r="D12" s="243" t="n">
         <v>-711657</v>
       </c>
-      <c r="E12" s="244" t="n">
-        <v>-0.023</v>
+      <c r="E12" s="244">
+        <f>D12/31537836</f>
+        <v/>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="125">
@@ -8559,8 +8568,9 @@
       <c r="D13" s="241" t="n">
         <v>112598</v>
       </c>
-      <c r="E13" s="242" t="n">
-        <v>0.004</v>
+      <c r="E13" s="242">
+        <f>D13/31537836</f>
+        <v/>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="125">
@@ -8580,8 +8590,9 @@
       <c r="D14" s="239" t="n">
         <v>31009</v>
       </c>
-      <c r="E14" s="240" t="n">
-        <v>0.001</v>
+      <c r="E14" s="240">
+        <f>D14/31537836</f>
+        <v/>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="125">
@@ -8601,8 +8612,9 @@
       <c r="D15" s="236" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="237" t="n">
-        <v>0</v>
+      <c r="E15" s="237">
+        <f>D15/31537836</f>
+        <v/>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="125">
@@ -8622,8 +8634,9 @@
       <c r="D16" s="243" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="244" t="n">
-        <v>0</v>
+      <c r="E16" s="244">
+        <f>D16/31537836</f>
+        <v/>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="125">
@@ -9434,22 +9447,25 @@
           <t>Founder salary</t>
         </is>
       </c>
-      <c r="B18" s="137" t="n">
-        <v>4396</v>
+      <c r="B18" s="137">
+        <f>Assumptions!B74/(12*Assumptions!$B$6)</f>
+        <v/>
       </c>
       <c r="C18" s="179">
         <f>B18/B10</f>
         <v/>
       </c>
-      <c r="D18" s="137" t="n">
-        <v>4396</v>
+      <c r="D18" s="137">
+        <f>Assumptions!B74/(12*Assumptions!$B$6)</f>
+        <v/>
       </c>
       <c r="E18" s="179">
         <f>D18/D10</f>
         <v/>
       </c>
-      <c r="F18" s="137" t="n">
-        <v>4396</v>
+      <c r="F18" s="137">
+        <f>Assumptions!B74/(12*Assumptions!$B$6)</f>
+        <v/>
       </c>
       <c r="G18" s="179">
         <f>F18/F10</f>
@@ -10379,16 +10395,16 @@
         </is>
       </c>
       <c r="B28" s="193">
-        <f>B27/8200</f>
+        <f>B27/B51</f>
         <v/>
       </c>
       <c r="C28" s="193">
-        <f>C27/8200</f>
+        <f>C27/B51</f>
         <v/>
       </c>
       <c r="D28" s="136" t="inlineStr">
         <is>
-          <t>Pre-revenue burn rate = ~EUR 9,725/mo</t>
+          <t>Seed / pre-revenue monthly burn</t>
         </is>
       </c>
       <c r="E28" s="127" t="n"/>
@@ -10724,7 +10740,7 @@
         </is>
       </c>
       <c r="B51" s="144" t="n">
-        <v>9725.274725274725</v>
+        <v>9725.27472527473</v>
       </c>
       <c r="C51" s="136" t="inlineStr">
         <is>
@@ -11118,11 +11134,11 @@
         </is>
       </c>
       <c r="B81" s="155">
-        <f>74*-3</f>
+        <f>-B74*3</f>
         <v/>
       </c>
       <c r="C81" s="155">
-        <f>74*-6</f>
+        <f>-C74*6</f>
         <v/>
       </c>
       <c r="D81" s="152" t="inlineStr">
@@ -11203,8 +11219,8 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A55:E55"/>
+    <mergeCell ref="B40:E40"/>
     <mergeCell ref="B41:E41"/>
-    <mergeCell ref="B40:E40"/>
     <mergeCell ref="A57:E57"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="B43:E43"/>
@@ -11372,9 +11388,16 @@
           <t>Annual OTA commissions paid</t>
         </is>
       </c>
-      <c r="B9" s="127" t="n"/>
+      <c r="B9" s="127">
+        <f>25000000*0.18*0.5</f>
+        <v/>
+      </c>
       <c r="C9" s="127" t="n"/>
-      <c r="D9" s="127" t="n"/>
+      <c r="D9" s="127" t="inlineStr">
+        <is>
+          <t>EUR 25M × 18% × 50% = EUR 2.25M</t>
+        </is>
+      </c>
       <c r="E9" s="127" t="n"/>
       <c r="F9" s="127" t="n"/>
       <c r="G9" s="127" t="n"/>
@@ -11406,9 +11429,16 @@
           <t>Annual savings from 5% shift</t>
         </is>
       </c>
-      <c r="B11" s="127" t="n"/>
+      <c r="B11" s="127">
+        <f>B9*0.05</f>
+        <v/>
+      </c>
       <c r="C11" s="127" t="n"/>
-      <c r="D11" s="127" t="n"/>
+      <c r="D11" s="127" t="inlineStr">
+        <is>
+          <t>5% × OTA commissions</t>
+        </is>
+      </c>
       <c r="E11" s="127" t="n"/>
       <c r="F11" s="127" t="n"/>
       <c r="G11" s="127" t="n"/>
@@ -11419,9 +11449,8 @@
           <t>Platform annual cost (low)</t>
         </is>
       </c>
-      <c r="B12" s="202">
-        <f>25000000*0.18*0.5</f>
-        <v/>
+      <c r="B12" s="202" t="n">
+        <v>30000</v>
       </c>
       <c r="C12" s="127" t="n"/>
       <c r="D12" s="136" t="inlineStr">
@@ -11439,10 +11468,8 @@
           <t>Platform annual cost (high)</t>
         </is>
       </c>
-      <c r="B13" s="202" t="inlineStr">
-        <is>
-          <t>EUR 60,000</t>
-        </is>
+      <c r="B13" s="202" t="n">
+        <v>60000</v>
       </c>
       <c r="C13" s="127" t="n"/>
       <c r="D13" s="136" t="inlineStr">
@@ -11461,11 +11488,15 @@
         </is>
       </c>
       <c r="B14" s="148">
-        <f>B11*0.05</f>
+        <f>B11/B12</f>
         <v/>
       </c>
       <c r="C14" s="127" t="n"/>
-      <c r="D14" s="127" t="n"/>
+      <c r="D14" s="127" t="inlineStr">
+        <is>
+          <t>Annual savings / platform cost (low)</t>
+        </is>
+      </c>
       <c r="E14" s="127" t="n"/>
       <c r="F14" s="127" t="n"/>
       <c r="G14" s="127" t="n"/>
@@ -11507,11 +11538,18 @@
         </is>
       </c>
       <c r="B17" s="203">
-        <f>112500/30000</f>
-        <v/>
-      </c>
-      <c r="C17" s="127" t="n"/>
-      <c r="D17" s="127" t="n"/>
+        <f>3000*12</f>
+        <v/>
+      </c>
+      <c r="C17" s="127">
+        <f>8000*12</f>
+        <v/>
+      </c>
+      <c r="D17" s="127" t="inlineStr">
+        <is>
+          <t>Monthly × 12</t>
+        </is>
+      </c>
       <c r="E17" s="127" t="n"/>
       <c r="F17" s="127" t="n"/>
       <c r="G17" s="127" t="n"/>
@@ -11560,10 +11598,7 @@
     </row>
     <row r="20" ht="19.5" customHeight="1" s="125">
       <c r="A20" s="127" t="n"/>
-      <c r="B20" s="187">
-        <f>5500*12</f>
-        <v/>
-      </c>
+      <c r="B20" s="187" t="n"/>
       <c r="C20" s="127" t="n"/>
       <c r="D20" s="127" t="n"/>
       <c r="E20" s="127" t="n"/>
@@ -12694,7 +12729,7 @@
       <c r="D19" s="127" t="n"/>
       <c r="E19" s="136" t="inlineStr">
         <is>
-          <t>50-75+ target</t>
+          <t>100-150 hotels (business plan target)</t>
         </is>
       </c>
       <c r="F19" s="127" t="n"/>
@@ -13445,18 +13480,19 @@
     <row r="29" ht="19.5" customHeight="1" s="125">
       <c r="A29" s="134" t="inlineStr">
         <is>
-          <t>G&amp;C: Cash capital (CHF 200K max)</t>
+          <t>G&amp;C: Cash capital (initial seed range)</t>
         </is>
       </c>
       <c r="B29" s="143" t="n">
-        <v>222222</v>
+        <v>164835</v>
       </c>
       <c r="C29" s="136" t="n">
         <v>4</v>
       </c>
-      <c r="D29" s="143">
-        <f>B29*C29</f>
-        <v/>
+      <c r="D29" s="143" t="inlineStr">
+        <is>
+          <t>Corrected seed anchor at CHF 150K / 0.91 FX</t>
+        </is>
       </c>
       <c r="E29" s="127" t="n"/>
       <c r="F29" s="127" t="n"/>
@@ -13728,15 +13764,15 @@
         </is>
       </c>
       <c r="B43" s="179">
-        <f>SUM(B38:B41)</f>
+        <f>SUM(B39:B42)</f>
         <v/>
       </c>
       <c r="C43" s="179">
-        <f>SUM(C38:C41)</f>
+        <f>SUM(C39:C42)</f>
         <v/>
       </c>
       <c r="D43" s="179">
-        <f>SUM(D38:D41)</f>
+        <f>SUM(D39:D42)</f>
         <v/>
       </c>
       <c r="E43" s="127" t="n"/>
@@ -16614,7 +16650,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="15" customHeight="1" s="125">
       <c r="A3" s="124" t="inlineStr">
         <is>
           <t>Source: research/synthetic-survey/run-2026-03-22-business-plan-monte-carlo-v2/</t>
@@ -17489,7 +17525,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="15" customHeight="1" s="125">
       <c r="A3" s="124" t="inlineStr">
         <is>
           <t>Source: research/synthetic-survey/run-2026-03-22-business-plan-monte-carlo-v2/</t>
@@ -17692,58 +17728,22 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="125">
-      <c r="A11" s="157" t="inlineStr">
-        <is>
-          <t>Month 48</t>
-        </is>
-      </c>
-      <c r="B11" s="215" t="n">
-        <v>254</v>
-      </c>
-      <c r="C11" s="215" t="n">
-        <v>320</v>
-      </c>
-      <c r="D11" s="215" t="n">
-        <v>342</v>
-      </c>
-      <c r="E11" s="215" t="n">
-        <v>362</v>
-      </c>
-      <c r="F11" s="215" t="n">
-        <v>391</v>
-      </c>
-      <c r="G11" s="157" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="A11" s="157" t="n"/>
+      <c r="B11" s="215" t="n"/>
+      <c r="C11" s="215" t="n"/>
+      <c r="D11" s="215" t="n"/>
+      <c r="E11" s="215" t="n"/>
+      <c r="F11" s="215" t="n"/>
+      <c r="G11" s="157" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="125">
-      <c r="A12" s="214" t="inlineStr">
-        <is>
-          <t>Month 60</t>
-        </is>
-      </c>
-      <c r="B12" s="216" t="n">
-        <v>318</v>
-      </c>
-      <c r="C12" s="216" t="n">
-        <v>332</v>
-      </c>
-      <c r="D12" s="216" t="n">
-        <v>358</v>
-      </c>
-      <c r="E12" s="216" t="n">
-        <v>426</v>
-      </c>
-      <c r="F12" s="216" t="n">
-        <v>498</v>
-      </c>
-      <c r="G12" s="214" t="inlineStr">
-        <is>
-          <t>+104</t>
-        </is>
-      </c>
+      <c r="A12" s="214" t="n"/>
+      <c r="B12" s="216" t="n"/>
+      <c r="C12" s="216" t="n"/>
+      <c r="D12" s="216" t="n"/>
+      <c r="E12" s="216" t="n"/>
+      <c r="F12" s="216" t="n"/>
+      <c r="G12" s="214" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="125">
       <c r="A14" s="163" t="inlineStr">
@@ -17931,31 +17931,13 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="125">
-      <c r="A21" s="157" t="inlineStr">
-        <is>
-          <t>Month 60</t>
-        </is>
-      </c>
-      <c r="B21" s="215" t="n">
-        <v>8618089</v>
-      </c>
-      <c r="C21" s="215" t="n">
-        <v>9849256</v>
-      </c>
-      <c r="D21" s="215" t="n">
-        <v>11557506</v>
-      </c>
-      <c r="E21" s="215" t="n">
-        <v>14162706</v>
-      </c>
-      <c r="F21" s="215" t="n">
-        <v>17354168</v>
-      </c>
-      <c r="G21" s="157" t="inlineStr">
-        <is>
-          <t>+32%</t>
-        </is>
-      </c>
+      <c r="A21" s="157" t="n"/>
+      <c r="B21" s="215" t="n"/>
+      <c r="C21" s="215" t="n"/>
+      <c r="D21" s="215" t="n"/>
+      <c r="E21" s="215" t="n"/>
+      <c r="F21" s="215" t="n"/>
+      <c r="G21" s="157" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="125">
       <c r="A23" s="163" t="inlineStr">
@@ -18292,7 +18274,7 @@
     <row r="39" ht="15" customHeight="1" s="125">
       <c r="A39" s="163" t="inlineStr">
         <is>
-          <t>MONTHLY P&amp;L SNAPSHOT (P50, EUR)</t>
+          <t>ILLUSTRATIVE MONTHLY P&amp;L SNAPSHOT (legacy exploratory build, not canonical path table)</t>
         </is>
       </c>
       <c r="B39" s="164" t="n"/>
@@ -18774,42 +18756,42 @@
     <row r="61" ht="15" customHeight="1" s="125">
       <c r="A61" s="211" t="inlineStr">
         <is>
-          <t>Same capital (CHF 200K seed), same team ceiling (8 people). Difference: 5 acquisition channels compound.</t>
+          <t>Same seed structure (CHF 120-150K initial capital) plus a milestone-based angel tranche. Difference: more support on onboarding, integrations, and group expansion.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="125">
       <c r="A62" s="211" t="inlineStr">
         <is>
-          <t>Network (Amedeo/Corsaro): ~3.5 intros/mo, 67% conv. Direct: founder 0.5/mo → sales team 3.5/mo.</t>
+          <t>Network remains the first channel. The upside comes from stronger expansion and follow-on distribution support, not a different wedge.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="125">
       <c r="A63" s="211" t="inlineStr">
         <is>
-          <t>PLG starts M18 (~4/mo). Channel partners M24 (~3/mo). Inbound M12 (~2.5/mo).</t>
+          <t>Additional execution capacity starts after traction, rather than assuming cold-volume scale from day one.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="125">
       <c r="A64" s="211" t="inlineStr">
         <is>
-          <t>Group rollouts (portfolio deals) add lumpiness: probability-weighted 2-5 hotels per event.</t>
+          <t>Group rollouts remain the main step-function driver in the upside path.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="125">
       <c r="A65" s="211" t="inlineStr">
         <is>
-          <t>M36 P50: 162 hotels, EUR 4.46M ARR — business plan target of 100-150 is between P10 and P50.</t>
+          <t>M36 P50: 154 hotels, EUR 5.33M ARR — this is the canonical follow-on-angel path used in the business plan.</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="125">
       <c r="A66" s="211" t="inlineStr">
         <is>
-          <t>M60 P50: 358 hotels, EUR 11.6M ARR, EUR 63.6M exit at 5.5x. Rev/employee: EUR 1.4M.</t>
+          <t>M60 P50: 321 hotels, EUR 13.22M ARR, EUR 68.1M exit at 5.15x.</t>
         </is>
       </c>
     </row>

</xml_diff>